<commit_message>
no-code bug fix (ner, nlu)
</commit_message>
<xml_diff>
--- a/sample_apps/lab_app_ja/lab_app_scenario_ja.xlsx
+++ b/sample_apps/lab_app_ja/lab_app_scenario_ja.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nakano\system\dialbb\dialbb-next\sample_apps\lab_app_ja\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nakano\system\dialbb\dialbb-main\sample_apps\lab_app_ja\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0B598DB-8B5F-4D13-9B82-7BE05D53628F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A44083F0-0AAE-41A0-A13D-7AD16A714299}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C3566FB2-A815-41D8-9347-99D11DD601B4}"/>
+    <workbookView xWindow="0" yWindow="368" windowWidth="21600" windowHeight="11054" xr2:uid="{C3566FB2-A815-41D8-9347-99D11DD601B4}"/>
   </bookViews>
   <sheets>
     <sheet name="scenario" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="88">
   <si>
     <t>system utterance</t>
     <phoneticPr fontId="1"/>
@@ -990,21 +990,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC9D1DC6-E066-4D71-9ECD-01107058A46B}">
-  <dimension ref="A1:H38"/>
-  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15"/>
+  <dimension ref="A1:H37"/>
+  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="8.5703125" style="9"/>
-    <col min="2" max="2" width="25.42578125" style="9" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="29.5703125" style="10" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.85546875" style="10" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="24.28515625" style="9" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="33.42578125" style="10" customWidth="1"/>
+    <col min="1" max="1" width="8.59765625" style="9"/>
+    <col min="2" max="2" width="25.3984375" style="9" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="29.59765625" style="10" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.86328125" style="10" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24.265625" style="9" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="33.3984375" style="10" customWidth="1"/>
     <col min="7" max="7" width="39" style="10" customWidth="1"/>
-    <col min="8" max="8" width="37.85546875" style="9" bestFit="1" customWidth="1"/>
-    <col min="9" max="16384" width="8.5703125" style="9"/>
+    <col min="8" max="8" width="37.86328125" style="9" bestFit="1" customWidth="1"/>
+    <col min="9" max="16384" width="8.59765625" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1" ht="30">
+    <row r="1" spans="1:8" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
@@ -1047,7 +1047,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:8" s="11" customFormat="1" ht="60">
+    <row r="3" spans="1:8" s="11" customFormat="1" ht="42.75">
       <c r="A3" s="11" t="s">
         <v>29</v>
       </c>
@@ -1083,7 +1083,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="5" spans="1:8" s="13" customFormat="1" ht="75">
+    <row r="5" spans="1:8" s="13" customFormat="1" ht="57">
       <c r="A5" s="13" t="s">
         <v>29</v>
       </c>
@@ -1093,11 +1093,19 @@
       <c r="C5" s="14" t="s">
         <v>85</v>
       </c>
-      <c r="D5" s="14"/>
+      <c r="D5" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" s="13" t="s">
+        <v>3</v>
+      </c>
       <c r="F5" s="14"/>
       <c r="G5" s="14"/>
-    </row>
-    <row r="6" spans="1:8" s="13" customFormat="1" ht="30">
+      <c r="H5" s="13" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" s="13" customFormat="1">
       <c r="A6" s="13" t="s">
         <v>29</v>
       </c>
@@ -1105,11 +1113,9 @@
         <v>54</v>
       </c>
       <c r="C6" s="14"/>
-      <c r="D6" s="14" t="s">
-        <v>12</v>
-      </c>
+      <c r="D6" s="14"/>
       <c r="E6" s="13" t="s">
-        <v>3</v>
+        <v>86</v>
       </c>
       <c r="F6" s="14"/>
       <c r="G6" s="14"/>
@@ -1125,17 +1131,19 @@
         <v>54</v>
       </c>
       <c r="C7" s="14"/>
-      <c r="D7" s="14"/>
+      <c r="D7" s="14" t="s">
+        <v>5</v>
+      </c>
       <c r="E7" s="13" t="s">
-        <v>86</v>
+        <v>13</v>
       </c>
       <c r="F7" s="14"/>
       <c r="G7" s="14"/>
       <c r="H7" s="13" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" s="13" customFormat="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" s="13" customFormat="1" ht="28.5">
       <c r="A8" s="13" t="s">
         <v>29</v>
       </c>
@@ -1143,58 +1151,58 @@
         <v>54</v>
       </c>
       <c r="C8" s="14"/>
-      <c r="D8" s="14" t="s">
-        <v>5</v>
-      </c>
-      <c r="E8" s="13" t="s">
-        <v>13</v>
-      </c>
+      <c r="D8" s="14"/>
       <c r="F8" s="14"/>
-      <c r="G8" s="14"/>
+      <c r="G8" s="14" t="s">
+        <v>71</v>
+      </c>
       <c r="H8" s="13" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" s="15" customFormat="1" ht="57">
+      <c r="A9" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="B9" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="C9" s="16" t="s">
+        <v>80</v>
+      </c>
+      <c r="D9" s="16" t="s">
+        <v>9</v>
+      </c>
+      <c r="E9" s="15" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" s="13" customFormat="1" ht="30">
-      <c r="A9" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="B9" s="13" t="s">
-        <v>54</v>
-      </c>
-      <c r="C9" s="14"/>
-      <c r="D9" s="14"/>
-      <c r="F9" s="14"/>
-      <c r="G9" s="14" t="s">
-        <v>71</v>
-      </c>
-      <c r="H9" s="13" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" s="15" customFormat="1" ht="75">
+      <c r="F9" s="16"/>
+      <c r="G9" s="16"/>
+      <c r="H9" s="15" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" s="15" customFormat="1">
       <c r="A10" s="15" t="s">
         <v>29</v>
       </c>
       <c r="B10" s="15" t="s">
         <v>55</v>
       </c>
-      <c r="C10" s="16" t="s">
-        <v>80</v>
-      </c>
+      <c r="C10" s="16"/>
       <c r="D10" s="16" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E10" s="15" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F10" s="16"/>
       <c r="G10" s="16"/>
       <c r="H10" s="15" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" s="15" customFormat="1" ht="30">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" s="15" customFormat="1">
       <c r="A11" s="15" t="s">
         <v>29</v>
       </c>
@@ -1203,18 +1211,18 @@
       </c>
       <c r="C11" s="16"/>
       <c r="D11" s="16" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="E11" s="15" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="F11" s="16"/>
       <c r="G11" s="16"/>
       <c r="H11" s="15" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" s="15" customFormat="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" s="15" customFormat="1" ht="28.5">
       <c r="A12" s="15" t="s">
         <v>29</v>
       </c>
@@ -1222,33 +1230,32 @@
         <v>55</v>
       </c>
       <c r="C12" s="16"/>
-      <c r="D12" s="16" t="s">
-        <v>5</v>
-      </c>
-      <c r="E12" s="15" t="s">
-        <v>13</v>
-      </c>
+      <c r="D12" s="16"/>
       <c r="F12" s="16"/>
-      <c r="G12" s="16"/>
+      <c r="G12" s="16" t="s">
+        <v>64</v>
+      </c>
       <c r="H12" s="15" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" s="1" customFormat="1">
+      <c r="A13" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D13" s="2"/>
+      <c r="F13" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="G13" s="2"/>
+      <c r="H13" s="1" t="s">
         <v>2</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" s="15" customFormat="1" ht="30">
-      <c r="A13" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="B13" s="15" t="s">
-        <v>55</v>
-      </c>
-      <c r="C13" s="16"/>
-      <c r="D13" s="16"/>
-      <c r="F13" s="16"/>
-      <c r="G13" s="16" t="s">
-        <v>64</v>
-      </c>
-      <c r="H13" s="15" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="14" spans="1:8" s="1" customFormat="1">
@@ -1258,54 +1265,57 @@
       <c r="B14" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="C14" s="2" t="s">
-        <v>75</v>
-      </c>
+      <c r="C14" s="2"/>
       <c r="D14" s="2"/>
       <c r="F14" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G14" s="2"/>
       <c r="H14" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" s="7" customFormat="1">
+      <c r="A15" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="B15" s="7" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="15" spans="1:8" s="1" customFormat="1">
-      <c r="A15" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="F15" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="G15" s="2"/>
-      <c r="H15" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" s="7" customFormat="1" ht="30">
+      <c r="C15" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="D15" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F15" s="8"/>
+      <c r="G15" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="H15" s="7" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" s="7" customFormat="1">
       <c r="A16" s="7" t="s">
         <v>29</v>
       </c>
       <c r="B16" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="C16" s="8" t="s">
-        <v>79</v>
-      </c>
+      <c r="C16" s="8"/>
       <c r="D16" s="8" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="F16" s="8"/>
       <c r="G16" s="8" t="s">
-        <v>73</v>
+        <v>52</v>
       </c>
       <c r="H16" s="7" t="s">
         <v>19</v>
@@ -1320,17 +1330,17 @@
       </c>
       <c r="C17" s="8"/>
       <c r="D17" s="8" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F17" s="8"/>
       <c r="G17" s="8" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="18" spans="1:8" s="7" customFormat="1">
@@ -1342,20 +1352,20 @@
       </c>
       <c r="C18" s="8"/>
       <c r="D18" s="8" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E18" s="7" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F18" s="8"/>
       <c r="G18" s="8" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H18" s="7" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="19" spans="1:8" s="7" customFormat="1" ht="30">
+    <row r="19" spans="1:8" s="7" customFormat="1">
       <c r="A19" s="7" t="s">
         <v>29</v>
       </c>
@@ -1364,67 +1374,69 @@
       </c>
       <c r="C19" s="8"/>
       <c r="D19" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="E19" s="7" t="s">
-        <v>21</v>
+        <v>33</v>
       </c>
       <c r="F19" s="8"/>
       <c r="G19" s="8" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" s="7" customFormat="1">
-      <c r="A20" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="B20" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="C20" s="8"/>
-      <c r="D20" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="F20" s="8"/>
-      <c r="G20" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="H20" s="7" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="21" spans="1:8" s="3" customFormat="1" ht="45">
-      <c r="A21" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="B21" s="3" t="s">
+    <row r="20" spans="1:8" s="3" customFormat="1" ht="28.5">
+      <c r="A20" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B20" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C21" s="4" t="s">
+      <c r="C20" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="D21" s="4" t="s">
+      <c r="D20" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="F21" s="4"/>
-      <c r="G21" s="4"/>
-      <c r="H21" s="3" t="s">
+      <c r="F20" s="4"/>
+      <c r="G20" s="4"/>
+      <c r="H20" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="22" spans="1:8" s="5" customFormat="1" ht="60">
+    <row r="21" spans="1:8" s="5" customFormat="1" ht="57">
+      <c r="A21" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="F21" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="G21" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="H21" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" s="5" customFormat="1" ht="28.5">
       <c r="A22" s="5" t="s">
         <v>29</v>
       </c>
       <c r="B22" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="C22" s="6" t="s">
-        <v>74</v>
-      </c>
+      <c r="C22" s="6"/>
       <c r="D22" s="6" t="s">
         <v>11</v>
       </c>
@@ -1432,251 +1444,249 @@
         <v>24</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="G22" s="6" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="H22" s="5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" s="5" customFormat="1" ht="45">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" s="5" customFormat="1">
       <c r="A23" s="5" t="s">
         <v>29</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>19</v>
+        <v>77</v>
       </c>
       <c r="C23" s="6"/>
-      <c r="D23" s="6" t="s">
-        <v>11</v>
-      </c>
+      <c r="D23" s="6"/>
       <c r="E23" s="5" t="s">
         <v>24</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="G23" s="6" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="H23" s="5" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" s="5" customFormat="1" ht="30">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" s="5" customFormat="1" ht="28.5">
       <c r="A24" s="5" t="s">
         <v>29</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>77</v>
-      </c>
-      <c r="C24" s="6"/>
-      <c r="D24" s="6"/>
-      <c r="E24" s="5" t="s">
-        <v>24</v>
+        <v>21</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="D24" s="6" t="s">
+        <v>26</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="G24" s="6" t="s">
-        <v>68</v>
-      </c>
+        <v>82</v>
+      </c>
+      <c r="G24" s="6"/>
       <c r="H24" s="5" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" s="5" customFormat="1" ht="30">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" s="5" customFormat="1">
       <c r="A25" s="5" t="s">
         <v>29</v>
       </c>
       <c r="B25" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="C25" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="D25" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="F25" s="6" t="s">
-        <v>82</v>
-      </c>
+      <c r="C25" s="6"/>
+      <c r="D25" s="6"/>
+      <c r="F25" s="6"/>
       <c r="G25" s="6"/>
       <c r="H25" s="5" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" s="5" customFormat="1">
-      <c r="A26" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="B26" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="C26" s="6"/>
-      <c r="D26" s="6"/>
-      <c r="F26" s="6"/>
-      <c r="G26" s="6"/>
-      <c r="H26" s="5" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="27" spans="1:8" s="1" customFormat="1" ht="45">
-      <c r="A27" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="B27" s="1" t="s">
+    <row r="26" spans="1:8" s="1" customFormat="1" ht="42.75">
+      <c r="A26" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B26" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="C27" s="2" t="s">
+      <c r="C26" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="D27" s="2"/>
-      <c r="F27" s="2"/>
-      <c r="G27" s="2"/>
-      <c r="H27" s="1" t="s">
+      <c r="D26" s="2"/>
+      <c r="F26" s="2"/>
+      <c r="G26" s="2"/>
+      <c r="H26" s="1" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="28" spans="1:8" s="3" customFormat="1" ht="30">
-      <c r="A28" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="B28" s="3" t="s">
+    <row r="27" spans="1:8" s="3" customFormat="1" ht="28.5">
+      <c r="A27" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B27" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="C28" s="4" t="s">
+      <c r="C27" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="D28" s="4"/>
-      <c r="F28" s="4"/>
-      <c r="G28" s="4"/>
-      <c r="H28" s="3" t="s">
+      <c r="D27" s="4"/>
+      <c r="F27" s="4"/>
+      <c r="G27" s="4"/>
+      <c r="H27" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="29" spans="1:8" s="1" customFormat="1" ht="45">
+    <row r="28" spans="1:8" s="1" customFormat="1" ht="42.75">
+      <c r="A28" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="F28" s="2"/>
+      <c r="G28" s="2"/>
+      <c r="H28" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" s="1" customFormat="1">
       <c r="A29" s="1" t="s">
         <v>29</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="C29" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="D29" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="E29" s="1" t="s">
-        <v>37</v>
-      </c>
+      <c r="C29" s="2"/>
+      <c r="D29" s="2"/>
       <c r="F29" s="2"/>
       <c r="G29" s="2"/>
       <c r="H29" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" s="7" customFormat="1" ht="28.5">
+      <c r="A30" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="B30" s="7" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="30" spans="1:8" s="1" customFormat="1">
-      <c r="A30" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="B30" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C30" s="2"/>
-      <c r="D30" s="2"/>
-      <c r="F30" s="2"/>
-      <c r="G30" s="2"/>
-      <c r="H30" s="1" t="s">
+      <c r="C30" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="D30" s="8"/>
+      <c r="F30" s="8"/>
+      <c r="G30" s="8"/>
+    </row>
+    <row r="31" spans="1:8" s="3" customFormat="1" ht="71.25">
+      <c r="A31" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="D31" s="4"/>
+      <c r="F31" s="4"/>
+      <c r="G31" s="4"/>
+    </row>
+    <row r="32" spans="1:8" s="5" customFormat="1" ht="327.75">
+      <c r="A32" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B32" s="5" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="31" spans="1:8" s="7" customFormat="1" ht="45">
-      <c r="A31" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="B31" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="C31" s="8" t="s">
-        <v>65</v>
-      </c>
-      <c r="D31" s="8"/>
-      <c r="F31" s="8"/>
-      <c r="G31" s="8"/>
-    </row>
-    <row r="32" spans="1:8" s="3" customFormat="1" ht="75">
-      <c r="A32" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="B32" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="C32" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="D32" s="4"/>
-      <c r="F32" s="4"/>
-      <c r="G32" s="4"/>
-    </row>
-    <row r="33" spans="1:8" s="5" customFormat="1" ht="360">
+      <c r="C32" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="D32" s="6"/>
+      <c r="F32" s="6"/>
+      <c r="G32" s="6"/>
+    </row>
+    <row r="33" spans="1:8" s="5" customFormat="1" ht="57">
       <c r="A33" s="5" t="s">
         <v>29</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>16</v>
+        <v>62</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>84</v>
+        <v>63</v>
       </c>
       <c r="D33" s="6"/>
       <c r="F33" s="6"/>
       <c r="G33" s="6"/>
     </row>
-    <row r="34" spans="1:8" s="5" customFormat="1" ht="75">
-      <c r="A34" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="B34" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="C34" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="D34" s="6"/>
-      <c r="F34" s="6"/>
-      <c r="G34" s="6"/>
-    </row>
-    <row r="35" spans="1:8" s="1" customFormat="1" ht="60">
-      <c r="A35" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="B35" s="1" t="s">
+    <row r="34" spans="1:8" s="1" customFormat="1" ht="42.75">
+      <c r="A34" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B34" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C35" s="2" t="s">
+      <c r="C34" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D35" s="2"/>
-      <c r="F35" s="2"/>
-      <c r="G35" s="2"/>
-    </row>
-    <row r="36" spans="1:8" s="5" customFormat="1" ht="60">
-      <c r="A36" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="B36" s="5" t="s">
+      <c r="D34" s="2"/>
+      <c r="F34" s="2"/>
+      <c r="G34" s="2"/>
+    </row>
+    <row r="35" spans="1:8" s="5" customFormat="1" ht="42.75">
+      <c r="A35" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B35" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="C36" s="6" t="s">
+      <c r="C35" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="D36" s="6"/>
-      <c r="F36" s="6"/>
-      <c r="G36" s="6"/>
+      <c r="D35" s="6"/>
+      <c r="F35" s="6"/>
+      <c r="G35" s="6"/>
+    </row>
+    <row r="36" spans="1:8" s="3" customFormat="1">
+      <c r="A36" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="D36" s="4"/>
+      <c r="E36" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F36" s="4"/>
+      <c r="G36" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="H36" s="3" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="37" spans="1:8" s="3" customFormat="1">
       <c r="A37" s="3" t="s">
@@ -1685,35 +1695,13 @@
       <c r="B37" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C37" s="4" t="s">
-        <v>45</v>
-      </c>
+      <c r="C37" s="4"/>
       <c r="D37" s="4"/>
-      <c r="E37" s="3" t="s">
-        <v>13</v>
-      </c>
       <c r="F37" s="4"/>
       <c r="G37" s="4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H37" s="3" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="38" spans="1:8" s="3" customFormat="1">
-      <c r="A38" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="B38" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="C38" s="4"/>
-      <c r="D38" s="4"/>
-      <c r="F38" s="4"/>
-      <c r="G38" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="H38" s="3" t="s">
         <v>46</v>
       </c>
     </row>

</xml_diff>